<commit_message>
docs: inventory bayesian parameter data needs
</commit_message>
<xml_diff>
--- a/docs/statistics/bayesian_parameter_collection_template.xlsx
+++ b/docs/statistics/bayesian_parameter_collection_template.xlsx
@@ -8,14 +8,15 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原子事实核验" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源观测统计" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="抽取准确率" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源依赖" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="案件族CPD" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="权威锚定复核" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型发布记录" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="枚举值" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数需求清单" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原子事实核验" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源观测统计" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="抽取准确率" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源依赖" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="案件族CPD" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="权威锚定复核" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型发布记录" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="枚举值" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="LabelValues">'枚举值'!$A$2:$A$4</definedName>
@@ -29,15 +30,17 @@
     <definedName name="CalibrationValues">'枚举值'!$I$2:$I$4</definedName>
     <definedName name="ApprovalValues">'枚举值'!$J$2:$J$5</definedName>
     <definedName name="PrivacyValues">'枚举值'!$K$2:$K$4</definedName>
+    <definedName name="YesNoDataValues">'枚举值'!$L$2:$L$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'填写说明'!$A$1:$C$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'原子事实核验'!$A$1:$L$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'来源观测统计'!$A$1:$Q$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'抽取准确率'!$A$1:$M$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源依赖'!$A$1:$K$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'案件族CPD'!$A$1:$O$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'权威锚定复核'!$A$1:$K$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'模型发布记录'!$A$1:$N$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'枚举值'!$A$1:$K$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'参数需求清单'!$A$1:$K$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'原子事实核验'!$A$1:$L$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'来源观测统计'!$A$1:$Q$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'抽取准确率'!$A$1:$M$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'来源依赖'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'案件族CPD'!$A$1:$O$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'权威锚定复核'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'模型发布记录'!$A$1:$N$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'枚举值'!$A$1:$L$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -646,7 +649,825 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>标签值</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>案件族</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>观测指标</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>是/否/未知</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>依赖复核</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>核验状态</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>有效性</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>适用范围</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>校准状态</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>审批状态</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>隐私检查</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>真实数据需求</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>真</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>conduct_result</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>真阳性率</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>独立</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>未开始</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>有效</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>符合</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>expert_prior_unvalidated</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>草稿</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>需要</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>假</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>property_taking</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>假阳性率</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>可能依赖</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>待复核</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>待核验</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>不符合</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>pilot_uncalibrated</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>待审批</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>建议</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>public_order</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>确认依赖</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>一致</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>已失效</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>待法律复核</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>validated</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>已批准</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>不通过</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>禁止</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>public_safety</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>已裁决</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>已拒绝</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="n"/>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>不用于真值率学习</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>status_duty</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="n"/>
+      <c r="L6" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>参数类别</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>模型ID</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>节点/谓词</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>参数名称</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>当前来源</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>是否需真实数据</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>所需统计量</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>估计方法</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>最小分组维度</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>法律边界</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>根节点先验</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>全部案件族</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>各根事实节点</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>prior</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>专家先验</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>建议</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>核验为真/假/未知的数量</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Beta后验或分层Beta</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>案件族×谓词×时间窗</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>不得解释为有罪概率</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>按月离线更新</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>条件分布</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>全部案件族</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>各派生事实节点</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>intercept/weights</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>专家先验</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>需要</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>每种父节点状态下子节点真/假/未知数</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>加权二项逻辑回归或Beta-CPT</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>模型版本×父节点组合</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>只推断事实要素</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>保留未校准标记</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>来源观测</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>证据融合</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>角色×谓词×立场</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>sensitivity/FPR</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>待统计</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>需要</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>TP/FP/FN/TN及未知数</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Beta-Binomial并进行分层收缩</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>来源类别×谓词×立场</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>不得按角色直接设固定可信度</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>小样本不得单独发布</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>抽取质量</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>抽取器</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>字段或谓词</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>precision/recall/F1</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>待统计</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>需要</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>TP/FP/FN/TN及未知数</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>混淆矩阵</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>抽取器版本×字段</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>只评价抽取准确性</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>不代表事实真实性</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>来源依赖</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>证据融合</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>来源组</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>dependency</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>人工规则</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>需要</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>共同来源、复制、转述和共同制作计数</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>分组去重或依赖模型</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>来源A×来源B×依赖类型</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>同源材料不得重复加权</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>先人工复核</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>权威锚定</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>权威校验</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>专业结论范围</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>validity/scope</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>法律和人工复核</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>不用于真值率学习</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>有效性、适用范围、替代或失效状态</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>确定性校验</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>文书类型×版本</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>只锚定专业范围内事实</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>普通否认不直接削弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>法律规则</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>规则引擎</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>年龄/数额/次数/抗辩/边界</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>threshold/rule</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>现行法律</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>禁止</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>不采集训练统计</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>确定性规则和人工法律审查</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>法域×生效时间</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>不得进入贝叶斯训练</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>版本化保存</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K8"/>
+  <dataValidations count="1">
+    <dataValidation sqref="F2:F501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="无效枚举值" error="请选择下拉列表中的值。" promptTitle="受控字段" prompt="请选择受控枚举值；未知不得填写为假。" type="list">
+      <formula1>=YesNoDataValues</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -773,7 +1594,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -927,7 +1748,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1048,7 +1869,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1144,7 +1965,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1284,7 +2105,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1380,7 +2201,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1495,306 +2316,4 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>标签值</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>案件族</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>观测指标</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>是/否/未知</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>依赖复核</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>核验状态</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>有效性</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>适用范围</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>校准状态</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>审批状态</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>隐私检查</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>真</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>conduct_result</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>真阳性率</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>独立</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>有效</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>符合</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>expert_prior_unvalidated</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>草稿</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>假</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>property_taking</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>假阳性率</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>可能依赖</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>待复核</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>待核验</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>不符合</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>pilot_uncalibrated</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>待审批</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>通过</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>未知</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>public_order</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>未知</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>确认依赖</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>一致</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>已失效</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>待法律复核</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>validated</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>已批准</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>不通过</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n"/>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>public_safety</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>未知</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>已裁决</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>未知</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="n"/>
-      <c r="I5" s="2" t="n"/>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>已拒绝</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>status_duty</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="n"/>
-      <c r="K6" s="2" t="n"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:K6"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: preserve evidence boundaries in bayesian inference
</commit_message>
<xml_diff>
--- a/docs/statistics/bayesian_parameter_collection_template.xlsx
+++ b/docs/statistics/bayesian_parameter_collection_template.xlsx
@@ -1723,11 +1723,11 @@
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="n"/>
       <c r="M2" s="3">
-        <f>IF(E2="真阳性率",K2+F2,IF(E2="假阳性率",K2+G2,""))</f>
+        <f>IF(OR(E2="",K2="",L2="",K2&lt;=0,L2&lt;=0),"",IF(E2="真阳性率",IF(F2="","",K2+F2),IF(E2="假阳性率",IF(G2="","",K2+G2),"")))</f>
         <v/>
       </c>
       <c r="N2" s="3">
-        <f>IF(E2="真阳性率",L2+H2,IF(E2="假阳性率",L2+I2,""))</f>
+        <f>IF(OR(E2="",K2="",L2="",K2&lt;=0,L2&lt;=0),"",IF(E2="真阳性率",IF(H2="","",L2+H2),IF(E2="假阳性率",IF(I2="","",L2+I2),"")))</f>
         <v/>
       </c>
       <c r="O2" s="3">

</xml_diff>